<commit_message>
Updated viewport with scaling selectors and updated coord system
</commit_message>
<xml_diff>
--- a/data_structure.xlsx
+++ b/data_structure.xlsx
@@ -413,137 +413,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>n_element</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>n_nodes</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>ncon1</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>ncon2</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ncon3</t>
         </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>NDU</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>dzero</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>v</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>[0.0, 0.0, 2.0, 2.0, 4.0]</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>[-1.0, -5.0, -5.0, -1.0, -1.0]</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>10000000000</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>[0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0]</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>3</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>[1, 2, 3, 4, 5]</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
-        <v>0.721</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Working Subdivision with + and - buttons
</commit_message>
<xml_diff>
--- a/data_structure.xlsx
+++ b/data_structure.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,19 +490,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="C2" t="n">
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -534,19 +534,19 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>0.004</v>
+        <v>0.01</v>
       </c>
       <c r="G3" t="n">
-        <v>0.006</v>
+        <v>0.01</v>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -562,19 +562,19 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0.007</v>
+        <v>0.02</v>
       </c>
       <c r="G4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -590,19 +590,19 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0055</v>
+        <v>0.00859</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0035</v>
+        <v>0.00547</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -618,19 +618,19 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>0.002</v>
+        <v>0.008670000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>0.003</v>
+        <v>0.004500000000000001</v>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
@@ -646,19 +646,19 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D7" t="n">
         <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0035</v>
+        <v>0.00821</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0005</v>
+        <v>0.00489</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -674,19 +674,19 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0.00625</v>
+        <v>0.008310000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>0.00225</v>
+        <v>0.004900000000000001</v>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -702,19 +702,19 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D9" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E9" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0045</v>
+        <v>0.008280000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>0.002</v>
+        <v>0.00493</v>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -730,19 +730,19 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D10" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F10" t="n">
-        <v>0.00525</v>
+        <v>0.014335</v>
       </c>
       <c r="G10" t="n">
-        <v>0.00075</v>
+        <v>0.00225</v>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
@@ -758,19 +758,19 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E11" t="n">
         <v>14</v>
       </c>
       <c r="F11" t="n">
-        <v>0.00475</v>
+        <v>0.004335</v>
       </c>
       <c r="G11" t="n">
-        <v>0.00475</v>
+        <v>0.00225</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -786,7 +786,7 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D12" t="n">
         <v>14</v>
@@ -795,10 +795,10 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0.003</v>
+        <v>0.01</v>
       </c>
       <c r="G12" t="n">
-        <v>0.004500000000000001</v>
+        <v>0</v>
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
@@ -814,19 +814,19 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D13" t="n">
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F13" t="n">
-        <v>0.00375</v>
+        <v>0.009105</v>
       </c>
       <c r="G13" t="n">
-        <v>0.00325</v>
+        <v>0.007445</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
@@ -842,19 +842,19 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F14" t="n">
-        <v>0.00275</v>
+        <v>0.005</v>
       </c>
       <c r="G14" t="n">
-        <v>0.00175</v>
+        <v>0.005</v>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
@@ -870,19 +870,19 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F15" t="n">
-        <v>0.001</v>
+        <v>0.004105</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0015</v>
+        <v>0.002445</v>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -898,19 +898,19 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D16" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>0.00175</v>
+        <v>0.00844</v>
       </c>
       <c r="G16" t="n">
-        <v>0.00025</v>
+        <v>0.004695</v>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -926,16 +926,20 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D17" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+        <v>18</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.009295000000000001</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.007735000000000001</v>
+      </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="n">
@@ -949,11 +953,21 @@
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="C18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" t="n">
+        <v>19</v>
+      </c>
+      <c r="E18" t="n">
+        <v>17</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.014295</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.002735</v>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="n">
@@ -967,11 +981,21 @@
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="C19" t="n">
+        <v>19</v>
+      </c>
+      <c r="D19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" t="n">
+        <v>9</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.005</v>
+      </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="n">
@@ -985,11 +1009,21 @@
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+      <c r="C20" t="n">
+        <v>17</v>
+      </c>
+      <c r="D20" t="n">
+        <v>9</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.008630000000000001</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.004985</v>
+      </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="n">
@@ -1003,11 +1037,21 @@
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+      <c r="C21" t="n">
+        <v>19</v>
+      </c>
+      <c r="D21" t="n">
+        <v>9</v>
+      </c>
+      <c r="E21" t="n">
+        <v>17</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.008400000000000001</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.005180000000000001</v>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="n">
@@ -1021,11 +1065,21 @@
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+      <c r="C22" t="n">
+        <v>6</v>
+      </c>
+      <c r="D22" t="n">
+        <v>20</v>
+      </c>
+      <c r="E22" t="n">
+        <v>12</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.00826</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.004895</v>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="n">
@@ -1039,11 +1093,21 @@
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+      <c r="C23" t="n">
+        <v>20</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" t="n">
+        <v>16</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.008490000000000001</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.004700000000000001</v>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="n">
@@ -1057,11 +1121,21 @@
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+      <c r="C24" t="n">
+        <v>12</v>
+      </c>
+      <c r="D24" t="n">
+        <v>16</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.008450000000000001</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.005185</v>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
@@ -1075,11 +1149,21 @@
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+      <c r="C25" t="n">
+        <v>20</v>
+      </c>
+      <c r="D25" t="n">
+        <v>16</v>
+      </c>
+      <c r="E25" t="n">
+        <v>12</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.008435000000000002</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.0052</v>
+      </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="n">
@@ -1093,11 +1177,21 @@
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="C26" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" t="n">
+        <v>21</v>
+      </c>
+      <c r="E26" t="n">
+        <v>22</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.008245000000000001</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.00491</v>
+      </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="n">
@@ -1111,11 +1205,21 @@
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+      <c r="C27" t="n">
+        <v>21</v>
+      </c>
+      <c r="D27" t="n">
+        <v>6</v>
+      </c>
+      <c r="E27" t="n">
+        <v>15</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.008295</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.004915000000000001</v>
+      </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="n">
@@ -1129,9 +1233,15 @@
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="C28" t="n">
+        <v>22</v>
+      </c>
+      <c r="D28" t="n">
+        <v>15</v>
+      </c>
+      <c r="E28" t="n">
+        <v>5</v>
+      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
@@ -1147,9 +1257,15 @@
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="C29" t="n">
+        <v>21</v>
+      </c>
+      <c r="D29" t="n">
+        <v>15</v>
+      </c>
+      <c r="E29" t="n">
+        <v>22</v>
+      </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
@@ -1165,9 +1281,15 @@
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="C30" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" t="n">
+        <v>23</v>
+      </c>
+      <c r="E30" t="n">
+        <v>19</v>
+      </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
@@ -1183,9 +1305,15 @@
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="C31" t="n">
+        <v>23</v>
+      </c>
+      <c r="D31" t="n">
+        <v>7</v>
+      </c>
+      <c r="E31" t="n">
+        <v>22</v>
+      </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
@@ -1198,6 +1326,486 @@
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="n">
+        <v>19</v>
+      </c>
+      <c r="D32" t="n">
+        <v>22</v>
+      </c>
+      <c r="E32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="n">
+        <v>23</v>
+      </c>
+      <c r="D33" t="n">
+        <v>22</v>
+      </c>
+      <c r="E33" t="n">
+        <v>19</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="n">
+        <v>8</v>
+      </c>
+      <c r="D34" t="n">
+        <v>24</v>
+      </c>
+      <c r="E34" t="n">
+        <v>25</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="n">
+        <v>24</v>
+      </c>
+      <c r="D35" t="n">
+        <v>4</v>
+      </c>
+      <c r="E35" t="n">
+        <v>20</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="n">
+        <v>25</v>
+      </c>
+      <c r="D36" t="n">
+        <v>20</v>
+      </c>
+      <c r="E36" t="n">
+        <v>6</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="n">
+        <v>24</v>
+      </c>
+      <c r="D37" t="n">
+        <v>20</v>
+      </c>
+      <c r="E37" t="n">
+        <v>25</v>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="n">
+        <v>7</v>
+      </c>
+      <c r="D38" t="n">
+        <v>26</v>
+      </c>
+      <c r="E38" t="n">
+        <v>21</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="n">
+        <v>26</v>
+      </c>
+      <c r="D39" t="n">
+        <v>8</v>
+      </c>
+      <c r="E39" t="n">
+        <v>25</v>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="n">
+        <v>21</v>
+      </c>
+      <c r="D40" t="n">
+        <v>25</v>
+      </c>
+      <c r="E40" t="n">
+        <v>6</v>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="n">
+        <v>26</v>
+      </c>
+      <c r="D41" t="n">
+        <v>25</v>
+      </c>
+      <c r="E41" t="n">
+        <v>21</v>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="n">
+        <v>8</v>
+      </c>
+      <c r="D42" t="n">
+        <v>26</v>
+      </c>
+      <c r="E42" t="n">
+        <v>24</v>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="n">
+        <v>26</v>
+      </c>
+      <c r="D43" t="n">
+        <v>7</v>
+      </c>
+      <c r="E43" t="n">
+        <v>23</v>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="n">
+        <v>24</v>
+      </c>
+      <c r="D44" t="n">
+        <v>23</v>
+      </c>
+      <c r="E44" t="n">
+        <v>4</v>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="n">
+        <v>26</v>
+      </c>
+      <c r="D45" t="n">
+        <v>23</v>
+      </c>
+      <c r="E45" t="n">
+        <v>24</v>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>